<commit_message>
Add SOH report for 2026-09-30
</commit_message>
<xml_diff>
--- a/reports/SOH_29_09_2026.xlsx
+++ b/reports/SOH_29_09_2026.xlsx
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1239</v>
+        <v>1213</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>-12</v>
+        <v>-20</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>81000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1418</v>
+        <v>1409</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>26500</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>954</v>
+        <v>944</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>51000</v>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>1392</v>
+        <v>1326</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>3000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>621</v>
+        <v>573</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>1176</v>
+        <v>1110</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>3000</v>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>8000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>1245</v>
+        <v>1241</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="E103" s="3" t="n">
         <v>4708</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>271</v>
+        <v>247</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>4708</v>
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E111" s="3" t="n">
         <v>25000</v>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="E116" s="3" t="n">
         <v>36000</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2450</v>
+        <v>2426</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>705</v>
+        <v>681</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>1001</v>
+        <v>998</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E182" s="3" t="n">
         <v>1</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -10382,7 +10382,7 @@
         </is>
       </c>
       <c r="D359" s="2" t="n">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E359" s="3" t="n">
         <v>16261</v>
@@ -15730,7 +15730,7 @@
         </is>
       </c>
       <c r="D550" s="2" t="n">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="E550" s="3" t="n">
         <v>13522</v>
@@ -17242,7 +17242,7 @@
         </is>
       </c>
       <c r="D604" s="2" t="n">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="E604" s="3" t="n">
         <v>8331</v>
@@ -17579,7 +17579,7 @@
         </is>
       </c>
       <c r="D616" s="2" t="n">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="E616" s="3" t="n">
         <v>12094</v>
@@ -18559,7 +18559,7 @@
         </is>
       </c>
       <c r="D651" s="2" t="n">
-        <v>922</v>
+        <v>916</v>
       </c>
       <c r="E651" s="3" t="n">
         <v>6417</v>
@@ -18615,7 +18615,7 @@
         </is>
       </c>
       <c r="D653" s="2" t="n">
-        <v>1229</v>
+        <v>1223</v>
       </c>
       <c r="E653" s="3" t="n">
         <v>11078</v>
@@ -20799,7 +20799,7 @@
         </is>
       </c>
       <c r="D731" s="2" t="n">
-        <v>546</v>
+        <v>534</v>
       </c>
       <c r="E731" s="3" t="n">
         <v>9641</v>
@@ -21751,7 +21751,7 @@
         </is>
       </c>
       <c r="D765" s="2" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E765" s="3" t="n">
         <v>6934</v>
@@ -23880,7 +23880,7 @@
         </is>
       </c>
       <c r="D841" s="2" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E841" s="3" t="n">
         <v>13122</v>
@@ -24497,7 +24497,7 @@
         </is>
       </c>
       <c r="D863" s="2" t="n">
-        <v>1415</v>
+        <v>1410</v>
       </c>
       <c r="E863" s="3" t="n">
         <v>8181</v>
@@ -24721,7 +24721,7 @@
         </is>
       </c>
       <c r="D871" s="2" t="n">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E871" s="3" t="n">
         <v>14083</v>
@@ -28308,7 +28308,7 @@
         </is>
       </c>
       <c r="D999" s="2" t="n">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="E999" s="3" t="n">
         <v>10871</v>
@@ -28868,7 +28868,7 @@
         </is>
       </c>
       <c r="D1019" s="2" t="n">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="E1019" s="3" t="n">
         <v>8060</v>
@@ -28924,7 +28924,7 @@
         </is>
       </c>
       <c r="D1021" s="2" t="n">
-        <v>2474</v>
+        <v>2469</v>
       </c>
       <c r="E1021" s="3" t="n">
         <v>8767</v>
@@ -32537,7 +32537,7 @@
         </is>
       </c>
       <c r="D1150" s="2" t="n">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E1150" s="3" t="n">
         <v>8325</v>
@@ -38137,7 +38137,7 @@
         </is>
       </c>
       <c r="D1350" s="2" t="n">
-        <v>1406</v>
+        <v>1394</v>
       </c>
       <c r="E1350" s="3" t="n">
         <v>14093</v>
@@ -38529,7 +38529,7 @@
         </is>
       </c>
       <c r="D1364" s="2" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E1364" s="3" t="n">
         <v>18059</v>
@@ -39873,7 +39873,7 @@
         </is>
       </c>
       <c r="D1412" s="2" t="n">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="E1412" s="3" t="n">
         <v>9036</v>

</xml_diff>